<commit_message>
adaptation for time reporting to IFS
</commit_message>
<xml_diff>
--- a/django_app/TimesheetSystem.xlsx
+++ b/django_app/TimesheetSystem.xlsx
@@ -1031,7 +1031,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J98"/>
+  <dimension ref="A1:J105"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="25.140625" customWidth="1" min="3" max="3"/>
@@ -5940,6 +5940,356 @@
       </c>
       <c r="J98" t="n">
         <v>2611</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>4410</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>CHYTIL BŘETISLAV</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>199288/K1</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>199288/K1 - MIL08B (Data hall) / Bouygues</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>VYCHYSTÁVÁNÍ</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>10:01:46</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>10:01:48</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>00:00:01</t>
+        </is>
+      </c>
+      <c r="J99" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>4420</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Jiří BRANDA</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>199159-B3 - 43776X1-63 - ARCHON Pila etap 2</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>199159-B3 - 43776X1-63 - ARCHON Pila etap 2 - ARCHON Pila etap 2</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>MANIPULACE</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>10:12:28</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>10:13:27</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>00:00:58</t>
+        </is>
+      </c>
+      <c r="J100" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>4410</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Břetislav CHYTIL</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>199288/K1</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>199288/K1 - MIL08B (Data hall) / Bouygues</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>VYCHYSTÁVÁNÍ</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>11:01:24</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>11:01:27</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>00:00:03</t>
+        </is>
+      </c>
+      <c r="J101" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>4410</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Břetislav CHYTIL</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>200530-K1 - 45649E1-54 - SIEGE METROPOLE GRENOBLE</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>200530-K1 - 45649E1-54 - SIEGE METROPOLE GRENOBLE - SIEGE METROPOLE GRENOBLE</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>MANIPULACE</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>11:01:42</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>11:02:59</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>00:01:17</t>
+        </is>
+      </c>
+      <c r="J102" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>4420</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Jiří BRANDA</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>198838-B2 - 43715X1-54 - PEPE SKI</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>198838-B2 - 43715X1-54 - PEPE SKI - PEPE SKI</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>BALENÍ</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>11:21:08</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>11:22:37</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>00:01:28</t>
+        </is>
+      </c>
+      <c r="J103" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>4420</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Jiří BRANDA</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>197189-A1 - 43449X1-52 - Parkpalette Lnneburg - PH Leuphana</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>197189-A1 - 43449X1-52 - Parkpalette Lnneburg - PH Leuphana - Parkpalette Lnneburg - PH Leuphana</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>BALENÍ</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>11:43:50</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>11:43:56</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>00:00:05</t>
+        </is>
+      </c>
+      <c r="J104" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>4420</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Jiří BRANDA</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>197171-K4 - 43290X1-51 - Sanem Warehouse</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>197171-K4 - 43290X1-51 - Sanem Warehouse - Sanem Warehouse</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>BALENÍ</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>11:44:40</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>11:44:56</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>00:00:16</t>
+        </is>
+      </c>
+      <c r="J105" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -6034,7 +6384,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H181"/>
+  <dimension ref="A1:H183"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.42578125" customWidth="1" min="3" max="3"/>
@@ -13284,6 +13634,86 @@
         <v>1133</v>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>4420</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>BRANDA JIŘÍ</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>SKLAD</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>09:13:56</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>09:13:58</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>00:00:01</t>
+        </is>
+      </c>
+      <c r="H182" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>4420</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>BRANDA JIŘÍ</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>SKLAD</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>15:19:22</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>15:20:47</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>00:01:25</t>
+        </is>
+      </c>
+      <c r="H183" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
stock scanner and admin dashboard updates
</commit_message>
<xml_diff>
--- a/django_app/TimesheetSystem.xlsx
+++ b/django_app/TimesheetSystem.xlsx
@@ -7284,7 +7284,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H188"/>
+  <dimension ref="A1:H189"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.42578125" customWidth="1" min="3" max="3"/>
@@ -14814,6 +14814,46 @@
         <v>0</v>
       </c>
     </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>4234</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Marek RYGAL</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>ADMINISTRATIVA</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>16:11:41</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>16:11:54</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>00:00:12</t>
+        </is>
+      </c>
+      <c r="H189" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>